<commit_message>
feat: upgrade to multi-company M&A platform with company switcher, custom target builder, and multi-model Excel generator
</commit_message>
<xml_diff>
--- a/output/valuation_model.xlsx
+++ b/output/valuation_model.xlsx
@@ -123,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -189,9 +189,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -202,9 +199,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -631,7 +625,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All figures in USD millions unless otherwise noted  |  Tesla 10-K Annual Reports (FY2021–FY2024), Analyst Consensus Estimates (FY2025E)</t>
+          <t>USD Millions ($M)</t>
         </is>
       </c>
     </row>
@@ -1390,16 +1384,16 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>3009</v>
+        <v>3220</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>3164</v>
+        <v>3220</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>3174</v>
+        <v>3220</v>
       </c>
       <c r="E42" s="13" t="n">
-        <v>3211</v>
+        <v>3220</v>
       </c>
       <c r="F42" s="13" t="n">
         <v>3220</v>
@@ -2212,165 +2206,185 @@
           <t>TSLA</t>
         </is>
       </c>
-      <c r="C5" s="23" t="n">
-        <v>949900</v>
-      </c>
-      <c r="D5" s="23" t="n">
-        <v>918900</v>
-      </c>
-      <c r="E5" s="24" t="n">
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="n">
         <v>8.140000000000001</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="23" t="n">
         <v>42.3</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="G5" s="23" t="n">
         <v>93.09999999999999</v>
       </c>
-      <c r="H5" s="25" t="n">
+      <c r="H5" s="24" t="n">
         <v>0.155</v>
       </c>
-      <c r="I5" s="25" t="n">
+      <c r="I5" s="24" t="n">
         <v>0.225</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>BYD Co.</t>
         </is>
       </c>
-      <c r="B6" s="27" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>BYDDY</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n">
-        <v>128500</v>
-      </c>
-      <c r="D6" s="28" t="n">
-        <v>135200</v>
-      </c>
-      <c r="E6" s="29" t="n">
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="n">
         <v>1.51</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="27" t="n">
         <v>12.4</v>
       </c>
-      <c r="G6" s="29" t="n">
+      <c r="G6" s="27" t="n">
         <v>18.5</v>
       </c>
-      <c r="H6" s="30" t="n">
+      <c r="H6" s="28" t="n">
         <v>0.23</v>
       </c>
-      <c r="I6" s="30" t="n">
+      <c r="I6" s="28" t="n">
         <v>0.195</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Rivian Automotive</t>
         </is>
       </c>
-      <c r="B7" s="27" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>RIVN</t>
         </is>
       </c>
-      <c r="C7" s="28" t="n">
-        <v>17800</v>
-      </c>
-      <c r="D7" s="28" t="n">
-        <v>21500</v>
-      </c>
-      <c r="E7" s="29" t="n">
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="n">
         <v>3.47</v>
       </c>
-      <c r="F7" s="27" t="inlineStr">
+      <c r="F7" s="26" t="inlineStr">
         <is>
           <t>N/M</t>
         </is>
       </c>
-      <c r="G7" s="27" t="inlineStr">
+      <c r="G7" s="26" t="inlineStr">
         <is>
           <t>N/M</t>
         </is>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="28" t="n">
         <v>0.52</v>
       </c>
-      <c r="I7" s="30" t="n">
+      <c r="I7" s="28" t="n">
         <v>-0.42</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Lucid Group</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>LCID</t>
         </is>
       </c>
-      <c r="C8" s="28" t="n">
-        <v>6900</v>
-      </c>
-      <c r="D8" s="28" t="n">
-        <v>8200</v>
-      </c>
-      <c r="E8" s="29" t="n">
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="n">
         <v>3.9</v>
       </c>
-      <c r="F8" s="27" t="inlineStr">
+      <c r="F8" s="26" t="inlineStr">
         <is>
           <t>N/M</t>
         </is>
       </c>
-      <c r="G8" s="27" t="inlineStr">
+      <c r="G8" s="26" t="inlineStr">
         <is>
           <t>N/M</t>
         </is>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="28" t="n">
         <v>0.35</v>
       </c>
-      <c r="I8" s="30" t="n">
+      <c r="I8" s="28" t="n">
         <v>-0.95</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Ford Motor Co.</t>
         </is>
       </c>
-      <c r="B9" s="27" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="C9" s="28" t="n">
-        <v>42300</v>
-      </c>
-      <c r="D9" s="28" t="n">
-        <v>98700</v>
-      </c>
-      <c r="E9" s="29" t="n">
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="n">
         <v>0.6</v>
       </c>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="27" t="n">
         <v>6.2</v>
       </c>
-      <c r="G9" s="29" t="n">
+      <c r="G9" s="27" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H9" s="28" t="n">
         <v>-0.02</v>
       </c>
-      <c r="I9" s="30" t="n">
+      <c r="I9" s="28" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -2382,86 +2396,86 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B13" s="31" t="inlineStr">
+      <c r="B13" s="29" t="inlineStr">
         <is>
           <t>Peer Median</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>Tesla Metric</t>
-        </is>
-      </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Target Metric</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
         <is>
           <t>Implied EV ($M)</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="E13" s="29" t="inlineStr">
         <is>
           <t>Implied Price</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="B14" s="33" t="n">
+      <c r="B14" s="31" t="n">
         <v>12.4</v>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="32" t="n">
         <v>21716</v>
       </c>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="32" t="n">
         <v>269278.4</v>
       </c>
-      <c r="E14" s="35" t="n">
+      <c r="E14" s="33" t="n">
         <v>93.25416149068323</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>EV/Revenue</t>
         </is>
       </c>
-      <c r="B15" s="33" t="n">
+      <c r="B15" s="31" t="n">
         <v>3.47</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="32" t="n">
         <v>112800</v>
       </c>
-      <c r="D15" s="34" t="n">
+      <c r="D15" s="32" t="n">
         <v>391416</v>
       </c>
-      <c r="E15" s="35" t="n">
+      <c r="E15" s="33" t="n">
         <v>131.1850931677019</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>P/E Ratio</t>
         </is>
       </c>
-      <c r="B16" s="33" t="n">
+      <c r="B16" s="31" t="n">
         <v>18.5</v>
       </c>
-      <c r="C16" s="34" t="n">
+      <c r="C16" s="32" t="n">
         <v>10200</v>
       </c>
-      <c r="D16" s="34" t="n">
+      <c r="D16" s="32" t="n">
         <v>188700</v>
       </c>
-      <c r="E16" s="35" t="n">
+      <c r="E16" s="33" t="n">
         <v>58.60248447204969</v>
       </c>
     </row>
@@ -2552,147 +2566,147 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>-2%</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="35" t="n">
         <v>73.92630976549599</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="C5" s="35" t="n">
         <v>68.28937155838973</v>
       </c>
-      <c r="D5" s="37" t="n">
+      <c r="D5" s="35" t="n">
         <v>63.52060578901772</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="36" t="n">
         <v>59.43466180937368</v>
       </c>
-      <c r="F5" s="37" t="n">
+      <c r="F5" s="35" t="n">
         <v>55.89542177909068</v>
       </c>
-      <c r="G5" s="37" t="n">
+      <c r="G5" s="35" t="n">
         <v>52.8006728010426</v>
       </c>
-      <c r="H5" s="37" t="n">
+      <c r="H5" s="35" t="n">
         <v>50.07216986834886</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>-1%</t>
         </is>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="35" t="n">
         <v>75.02456943269814</v>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="C6" s="35" t="n">
         <v>69.27030106885728</v>
       </c>
-      <c r="D6" s="37" t="n">
+      <c r="D6" s="35" t="n">
         <v>64.40263880507224</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="E6" s="36" t="n">
         <v>60.23228815380083</v>
       </c>
-      <c r="F6" s="37" t="n">
+      <c r="F6" s="35" t="n">
         <v>56.62023522823889</v>
       </c>
-      <c r="G6" s="37" t="n">
+      <c r="G6" s="35" t="n">
         <v>53.46209265649079</v>
       </c>
-      <c r="H6" s="37" t="n">
+      <c r="H6" s="35" t="n">
         <v>50.6779510395247</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>+0%</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="36" t="n">
         <v>76.10948692630923</v>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="36" t="n">
         <v>70.23887333989329</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="36" t="n">
         <v>65.27315309319144</v>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E7" s="38" t="n">
         <v>61.01911897107111</v>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="36" t="n">
         <v>57.33488389290199</v>
       </c>
-      <c r="G7" s="38" t="n">
+      <c r="G7" s="36" t="n">
         <v>54.11390317655004</v>
       </c>
-      <c r="H7" s="38" t="n">
+      <c r="H7" s="36" t="n">
         <v>51.27461617423353</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>+1%</t>
         </is>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="B8" s="35" t="n">
         <v>77.17923530037638</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="C8" s="35" t="n">
         <v>71.19343600163121</v>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="35" t="n">
         <v>66.13064371694287</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E8" s="36" t="n">
         <v>61.79377541616126</v>
       </c>
-      <c r="F8" s="37" t="n">
+      <c r="F8" s="35" t="n">
         <v>58.0380979371487</v>
       </c>
-      <c r="G8" s="37" t="n">
+      <c r="G8" s="35" t="n">
         <v>54.7549296505984</v>
       </c>
-      <c r="H8" s="37" t="n">
+      <c r="H8" s="35" t="n">
         <v>51.86107425176072</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>+2%</t>
         </is>
       </c>
-      <c r="B9" s="37" t="n">
+      <c r="B9" s="35" t="n">
         <v>78.23192785628841</v>
       </c>
-      <c r="C9" s="37" t="n">
+      <c r="C9" s="35" t="n">
         <v>72.13228281311267</v>
       </c>
-      <c r="D9" s="37" t="n">
+      <c r="D9" s="35" t="n">
         <v>66.9735568311351</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="36" t="n">
         <v>62.55483397497813</v>
       </c>
-      <c r="F9" s="37" t="n">
+      <c r="F9" s="35" t="n">
         <v>58.72856651738545</v>
       </c>
-      <c r="G9" s="37" t="n">
+      <c r="G9" s="35" t="n">
         <v>55.38395955187245</v>
       </c>
-      <c r="H9" s="37" t="n">
+      <c r="H9" s="35" t="n">
         <v>52.43619923985318</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="41" t="inlineStr">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>Current Market Price: $295.00</t>
         </is>

</xml_diff>